<commit_message>
Export Data S26 (junction-pair corroboration) and regenerate supplement
assemble_supp_tables.py: junction_pair_table() writes
tableS40_junction_pair_corroboration.csv (260 pair-region rows) from the
Figure 6c primary_pair_results.
build_supplementary_data.py: s-junction-pairs added between s-longread
and s-psi-junctions; former Data S26/S27 become S27/S28.
Regenerated manuscript_supplement tree (Tables S1-S9, Data S1-S28) with
the copy-edited legends read from the manuscript supplement.
</commit_message>
<xml_diff>
--- a/manuscript/_m/manuscript_supplement/supplementary_data/dataS01_cohort_description.xlsx
+++ b/manuscript/_m/manuscript_supplement/supplementary_data/dataS01_cohort_description.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>One row per analysis (17 analyses over 16 region-level cohorts; the BrainSEQ schizophrenia caudate analysis includes the 238 control donors of the aging caudate analysis). Each donor contributes one sample per analysis. Age is in years; GTEx exact age is released top-coded at 70. BrainSEQ reports postmortem interval (PMI, h) and GTEx tissue ischemic time (min). Genes and transcripts are counts after the bundle expression filter, before the prevalence filter applied at module fitting. The CSV adds library kit, self-reported ancestry, manner of death or Hardy scale, feature counts before filtering and the snRNA-seq reference used for MuSiC deconvolution.</t>
+          <t>One row per analysis (17 analyses over 16 region-level cohorts; the BrainSEQ schizophrenia caudate analysis includes the 238 control donors of the aging caudate analysis). Each donor contributes one sample per analysis. Age is in years; Genotype-Tissue Expression (GTEx) exact age is released top-coded at 70. BrainSEQ reports postmortem interval (PMI, h) and GTEx tissue ischemic time (min). Genes and transcripts are counts after the bundle expression filter, before the prevalence filter applied at module fitting. The CSV adds library kit, self-reported ancestry, manner of death or Hardy scale, feature counts before filtering, and the single-nucleus RNA-sequencing (snRNA-seq) reference used for MuSiC deconvolution.</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 by manuscript/_h/build_supplementary_data.py</t>
+          <t>2026-10-04 by manuscript/_h/build_supplementary_data.py</t>
         </is>
       </c>
     </row>

</xml_diff>